<commit_message>
add inventory movements file
</commit_message>
<xml_diff>
--- a/Project-FTO/CO_2026.xlsx
+++ b/Project-FTO/CO_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtinoco2\Downloads\Failures-PMI\Project-FTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{463FE844-F9E0-4BC6-9D73-E803EEACBF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33449EB-CD32-4A5E-8234-A977D149A1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45DDE3C2-CA09-4F3B-B8A7-AA0F2A1ADE2F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="212">
   <si>
     <t>Máquina</t>
   </si>
@@ -206,9 +206,6 @@
     <t>1/23/2026</t>
   </si>
   <si>
-    <t>Marco</t>
-  </si>
-  <si>
     <t>Atoramiento capsula deforme 20.A730</t>
   </si>
   <si>
@@ -608,9 +605,6 @@
     <t>3/31/2026</t>
   </si>
   <si>
-    <t>Eduardo</t>
-  </si>
-  <si>
     <t>Si</t>
   </si>
   <si>
@@ -678,9 +672,6 @@
   </si>
   <si>
     <t>Tomar en cuenta el tiempo de rutinas y reparacion de DH</t>
-  </si>
-  <si>
-    <t>Milron</t>
   </si>
   <si>
     <t>Electrico realiza calibracion de gomas. Reparacion de DH en las ruedas HCI. 45 min por CO y 7 min por calibracion gomas</t>
@@ -1669,7 +1660,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>49</v>
@@ -1684,10 +1675,10 @@
         <v>1</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="K11" s="2">
         <v>60</v>
@@ -1716,7 +1707,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C12" s="3">
         <v>4</v>
@@ -1737,7 +1728,7 @@
         <v>0.66</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>24</v>
@@ -1773,10 +1764,10 @@
         <v>6</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>45</v>
@@ -1788,7 +1779,7 @@
         <v>0.66</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>24</v>
@@ -1826,7 +1817,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>45</v>
@@ -1873,19 +1864,19 @@
         <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" s="3">
         <v>7</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>22</v>
@@ -1894,7 +1885,7 @@
         <v>0.66</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>24</v>
@@ -1932,13 +1923,13 @@
         <v>7</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>22</v>
@@ -1947,10 +1938,10 @@
         <v>1</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="K16" s="2">
         <v>75</v>
@@ -2000,7 +1991,7 @@
         <v>0.66</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>24</v>
@@ -2032,7 +2023,7 @@
         <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C18" s="3">
         <v>8</v>
@@ -2041,7 +2032,7 @@
         <v>26</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>31</v>
@@ -2081,19 +2072,19 @@
         <v>29</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19" s="3">
         <v>8</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>22</v>
@@ -2102,7 +2093,7 @@
         <v>0.66</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>24</v>
@@ -2134,13 +2125,13 @@
         <v>35</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" s="3">
         <v>8</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>49</v>
@@ -2155,7 +2146,7 @@
         <v>0.66</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>24</v>
@@ -2187,7 +2178,7 @@
         <v>35</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C21" s="3">
         <v>8</v>
@@ -2199,7 +2190,7 @@
         <v>42</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>22</v>
@@ -2208,7 +2199,7 @@
         <v>0.66</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>24</v>
@@ -2240,7 +2231,7 @@
         <v>35</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="3">
         <v>9</v>
@@ -2261,7 +2252,7 @@
         <v>0.66</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>24</v>
@@ -2302,7 +2293,7 @@
         <v>19</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>20</v>
@@ -2358,7 +2349,7 @@
         <v>20</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>22</v>
@@ -2367,10 +2358,10 @@
         <v>1</v>
       </c>
       <c r="I24" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="K24" s="2">
         <v>90</v>
@@ -2408,7 +2399,7 @@
         <v>19</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>20</v>
@@ -2458,7 +2449,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>30</v>
@@ -2511,7 +2502,7 @@
         <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>31</v>
@@ -2564,13 +2555,13 @@
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>22</v>
@@ -2579,10 +2570,10 @@
         <v>1</v>
       </c>
       <c r="I28" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="K28" s="2">
         <v>60</v>
@@ -2617,13 +2608,13 @@
         <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>31</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>22</v>
@@ -2632,10 +2623,10 @@
         <v>1</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="K29" s="2">
         <v>60</v>
@@ -2676,7 +2667,7 @@
         <v>42</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>22</v>
@@ -2685,10 +2676,10 @@
         <v>1</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="K30" s="2">
         <v>45</v>
@@ -2717,19 +2708,19 @@
         <v>25</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" s="3">
         <v>8</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>22</v>
@@ -2738,10 +2729,10 @@
         <v>1</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K31" s="2">
         <v>60</v>
@@ -2770,19 +2761,19 @@
         <v>25</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C32" s="3">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="F32" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>22</v>
@@ -2791,10 +2782,10 @@
         <v>1</v>
       </c>
       <c r="I32" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J32" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="K32" s="2">
         <v>125</v>
@@ -2829,13 +2820,13 @@
         <v>7</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="F33" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>22</v>
@@ -2844,7 +2835,7 @@
         <v>0.66</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>24</v>
@@ -2870,7 +2861,7 @@
         <v>35</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C34" s="3">
         <v>9</v>
@@ -2891,7 +2882,7 @@
         <v>0.66</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>24</v>
@@ -2923,7 +2914,7 @@
         <v>17</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C35" s="3">
         <v>9</v>
@@ -2932,10 +2923,10 @@
         <v>19</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>22</v>
@@ -2944,7 +2935,7 @@
         <v>0.66</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>24</v>
@@ -2976,7 +2967,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C36" s="3">
         <v>9</v>
@@ -2988,7 +2979,7 @@
         <v>39</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>22</v>
@@ -2997,10 +2988,10 @@
         <v>1</v>
       </c>
       <c r="I36" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J36" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="K36" s="2">
         <v>45</v>
@@ -3035,10 +3026,10 @@
         <v>10</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>42</v>
@@ -3050,7 +3041,7 @@
         <v>1</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>47</v>
@@ -3091,7 +3082,7 @@
         <v>19</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>21</v>
@@ -3103,10 +3094,10 @@
         <v>1</v>
       </c>
       <c r="I38" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J38" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="K38" s="2">
         <v>45</v>
@@ -3156,7 +3147,7 @@
         <v>0.66</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>24</v>
@@ -3188,19 +3179,19 @@
         <v>29</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C40" s="3">
         <v>8</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>22</v>
@@ -3209,7 +3200,7 @@
         <v>0.66</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>24</v>
@@ -3250,7 +3241,7 @@
         <v>41</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>45</v>
@@ -3262,10 +3253,10 @@
         <v>1</v>
       </c>
       <c r="I41" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="K41" s="2">
         <v>60</v>
@@ -3306,7 +3297,7 @@
         <v>49</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>22</v>
@@ -3315,10 +3306,10 @@
         <v>1</v>
       </c>
       <c r="I42" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J42" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="K42" s="2">
         <v>45</v>
@@ -3359,7 +3350,7 @@
         <v>21</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>22</v>
@@ -3368,7 +3359,7 @@
         <v>1</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J43" s="2"/>
       <c r="K43" s="2">
@@ -3408,7 +3399,7 @@
         <v>39</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>22</v>
@@ -3417,10 +3408,10 @@
         <v>1</v>
       </c>
       <c r="I44" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="J44" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="K44" s="2">
         <v>45</v>
@@ -3446,7 +3437,7 @@
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B45" s="6">
         <v>46359</v>
@@ -3455,13 +3446,13 @@
         <v>11</v>
       </c>
       <c r="D45" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>22</v>
@@ -3497,7 +3488,7 @@
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B46" s="6">
         <v>46329</v>
@@ -3506,13 +3497,13 @@
         <v>11</v>
       </c>
       <c r="D46" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>22</v>
@@ -3521,7 +3512,7 @@
         <v>0.66</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>24</v>
@@ -3548,7 +3539,7 @@
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B47" s="6">
         <v>46115</v>
@@ -3557,13 +3548,13 @@
         <v>10</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E47" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>22</v>
@@ -3572,7 +3563,7 @@
         <v>0.66</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>24</v>
@@ -3601,22 +3592,22 @@
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C48" s="3">
         <v>8</v>
       </c>
       <c r="D48" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="F48" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>22</v>
@@ -3625,7 +3616,7 @@
         <v>0.66</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>24</v>
@@ -3652,7 +3643,7 @@
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B49" s="6">
         <v>46329</v>
@@ -3664,7 +3655,7 @@
         <v>41</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>42</v>
@@ -3676,10 +3667,10 @@
         <v>1</v>
       </c>
       <c r="I49" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J49" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="K49" s="2">
         <v>60</v>
@@ -3705,10 +3696,10 @@
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C50" s="3">
         <v>11</v>
@@ -3729,10 +3720,10 @@
         <v>1</v>
       </c>
       <c r="I50" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J50" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="K50" s="2">
         <v>60</v>
@@ -3758,16 +3749,16 @@
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C51" s="3">
         <v>12</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>49</v>
@@ -3782,10 +3773,10 @@
         <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K51" s="2">
         <v>40</v>
@@ -3814,7 +3805,7 @@
         <v>35</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C52" s="3">
         <v>12</v>
@@ -3835,10 +3826,10 @@
         <v>1</v>
       </c>
       <c r="I52" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J52" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="K52" s="2">
         <v>40</v>
@@ -3876,7 +3867,7 @@
         <v>33</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>21</v>
@@ -3912,7 +3903,7 @@
         <v>-0.56000000000000005</v>
       </c>
       <c r="Q53" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.35">
@@ -3920,7 +3911,7 @@
         <v>29</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C54" s="3">
         <v>11</v>
@@ -3929,7 +3920,7 @@
         <v>26</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>31</v>
@@ -3970,10 +3961,10 @@
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C55" s="3">
         <v>12</v>
@@ -3982,10 +3973,10 @@
         <v>37</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>22</v>
@@ -3994,10 +3985,10 @@
         <v>1</v>
       </c>
       <c r="I55" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="J55" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="K55" s="2">
         <v>40</v>
@@ -4023,10 +4014,10 @@
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C56" s="3">
         <v>12</v>
@@ -4038,7 +4029,7 @@
         <v>45</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>22</v>
@@ -4047,10 +4038,10 @@
         <v>1</v>
       </c>
       <c r="I56" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="J56" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="K56" s="2">
         <v>40</v>
@@ -4079,16 +4070,16 @@
         <v>29</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C57" s="3">
         <v>12</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>21</v>
@@ -4132,19 +4123,19 @@
         <v>29</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C58" s="3">
         <v>12</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>22</v>
@@ -4185,16 +4176,16 @@
         <v>29</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C59" s="3">
         <v>12</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>21</v>
@@ -4238,7 +4229,7 @@
         <v>29</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C60" s="3">
         <v>12</v>
@@ -4250,7 +4241,7 @@
         <v>21</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>22</v>
@@ -4259,7 +4250,7 @@
         <v>0.66</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J60" s="2" t="s">
         <v>24</v>
@@ -4288,22 +4279,22 @@
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C61" s="3">
         <v>12</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E61" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F61" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>22</v>
@@ -4312,7 +4303,7 @@
         <v>0.66</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J61" s="2" t="s">
         <v>24</v>
@@ -4341,22 +4332,22 @@
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C62" s="3">
         <v>12</v>
       </c>
       <c r="D62" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>22</v>
@@ -4365,10 +4356,10 @@
         <v>1</v>
       </c>
       <c r="I62" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J62" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="J62" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="K62" s="2">
         <v>60</v>
@@ -4394,22 +4385,22 @@
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C63" s="3">
         <v>12</v>
       </c>
       <c r="D63" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E63" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="F63" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>22</v>
@@ -4447,22 +4438,22 @@
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C64" s="3">
         <v>12</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>22</v>
@@ -4471,10 +4462,10 @@
         <v>1</v>
       </c>
       <c r="I64" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="J64" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="J64" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="K64" s="2">
         <v>60</v>
@@ -4500,10 +4491,10 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C65" s="3">
         <v>13</v>
@@ -4515,7 +4506,7 @@
         <v>49</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>22</v>
@@ -4524,10 +4515,10 @@
         <v>1</v>
       </c>
       <c r="I65" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="J65" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="K65" s="2">
         <v>40</v>
@@ -4553,16 +4544,16 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C66" s="3">
         <v>13</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>45</v>
@@ -4577,7 +4568,7 @@
         <v>0.66</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J66" s="2" t="s">
         <v>24</v>
@@ -4604,19 +4595,19 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C67" s="3">
         <v>13</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F67" s="2">
         <v>33.124000000000002</v>
@@ -4628,10 +4619,10 @@
         <v>1</v>
       </c>
       <c r="I67" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="J67" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="K67" s="2">
         <v>55</v>
@@ -4660,7 +4651,7 @@
         <v>35</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C68" s="3">
         <v>13</v>
@@ -4669,7 +4660,7 @@
         <v>37</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>45</v>
@@ -4681,7 +4672,7 @@
         <v>0.66</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>24</v>
@@ -4713,7 +4704,7 @@
         <v>29</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C69" s="3">
         <v>13</v>
@@ -4725,7 +4716,7 @@
         <v>31</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>22</v>
@@ -4766,7 +4757,7 @@
         <v>29</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C70" s="3">
         <v>13</v>
@@ -4775,10 +4766,10 @@
         <v>26</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>22</v>
@@ -4787,10 +4778,10 @@
         <v>1</v>
       </c>
       <c r="I70" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="J70" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="K70" s="2">
         <v>50</v>
@@ -4819,31 +4810,31 @@
         <v>29</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C71" s="3">
         <v>14</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>189</v>
+        <v>88</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>31</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H71" s="7">
         <v>1</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J71" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K71" s="2">
         <v>50</v>
@@ -4872,7 +4863,7 @@
         <v>29</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C72" s="3">
         <v>14</v>
@@ -4881,10 +4872,10 @@
         <v>26</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>22</v>
@@ -4893,7 +4884,7 @@
         <v>0.66</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>24</v>
@@ -4922,7 +4913,7 @@
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B73" s="6">
         <v>46207</v>
@@ -4931,13 +4922,13 @@
         <v>15</v>
       </c>
       <c r="D73" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>22</v>
@@ -4946,7 +4937,7 @@
         <v>0.66</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>24</v>
@@ -4984,13 +4975,13 @@
         <v>15</v>
       </c>
       <c r="D74" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E74" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E74" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="F74" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>22</v>
@@ -4999,7 +4990,7 @@
         <v>0.66</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>24</v>
@@ -5028,7 +5019,7 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B75" s="6">
         <v>46207</v>
@@ -5037,13 +5028,13 @@
         <v>15</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>42</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>22</v>
@@ -5052,7 +5043,7 @@
         <v>0.66</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="J75" s="2" t="s">
         <v>24</v>
@@ -5081,7 +5072,7 @@
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B76" s="6">
         <v>46269</v>
@@ -5090,10 +5081,10 @@
         <v>15</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>38</v>
@@ -5105,7 +5096,7 @@
         <v>0.66</v>
       </c>
       <c r="I76" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>24</v>
@@ -5134,7 +5125,7 @@
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B77" s="6">
         <v>46330</v>
@@ -5158,10 +5149,10 @@
         <v>1</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="J77" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K77" s="2">
         <v>40</v>
@@ -5190,19 +5181,19 @@
         <v>25</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C78" s="3">
         <v>14</v>
       </c>
       <c r="D78" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="G78" s="2" t="s">
         <v>22</v>
@@ -5240,7 +5231,7 @@
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B79" s="6">
         <v>46330</v>
@@ -5249,13 +5240,13 @@
         <v>15</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>22</v>
@@ -5264,10 +5255,10 @@
         <v>1</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K79" s="2">
         <v>55</v>
@@ -5302,13 +5293,13 @@
         <v>15</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>22</v>
@@ -5317,10 +5308,10 @@
         <v>1</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="J80" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K80" s="2">
         <v>65</v>
@@ -5349,13 +5340,13 @@
         <v>35</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C81" s="3">
         <v>16</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>39</v>
@@ -5370,10 +5361,10 @@
         <v>1</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K81" s="2">
         <v>40</v>
@@ -5408,13 +5399,13 @@
         <v>10</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>213</v>
+        <v>19</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>22</v>
@@ -5423,7 +5414,7 @@
         <v>0.66</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="J82" s="2" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
add commit file for capsules
</commit_message>
<xml_diff>
--- a/Project-FTO/CO_2026.xlsx
+++ b/Project-FTO/CO_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtinoco2\Downloads\Failures-PMI\Project-FTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33449EB-CD32-4A5E-8234-A977D149A1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FB7EC0-9283-48E2-98F3-DFA3C9B5A2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45DDE3C2-CA09-4F3B-B8A7-AA0F2A1ADE2F}"/>
   </bookViews>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>18</v>

</xml_diff>